<commit_message>
Update real-time sent status in CRM database
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -524,10 +524,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -576,10 +574,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -628,10 +624,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K4" t="b">
+        <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -685,10 +679,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K5" t="b">
+        <v>0</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -742,10 +734,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K6" t="b">
+        <v>0</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -799,10 +789,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K7" t="b">
+        <v>0</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -856,10 +844,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K8" t="b">
+        <v>0</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -913,10 +899,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K9" t="b">
+        <v>0</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -970,10 +954,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1022,10 +1004,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K11" t="b">
+        <v>0</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1079,10 +1059,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K12" t="b">
+        <v>0</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1136,10 +1114,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K13" t="b">
+        <v>0</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1193,10 +1169,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K14" t="b">
+        <v>0</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1250,10 +1224,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1302,10 +1274,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K16" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1354,10 +1324,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K17" t="b">
+        <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1416,10 +1384,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K18" t="b">
+        <v>0</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1478,10 +1444,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K19" t="b">
+        <v>0</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1535,10 +1499,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K20" t="b">
+        <v>0</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1592,10 +1554,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K21" t="b">
+        <v>0</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1649,10 +1609,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K22" t="b">
+        <v>0</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1706,10 +1664,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K23" t="b">
+        <v>0</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1763,10 +1719,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K24" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1815,10 +1769,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K25" t="b">
+        <v>0</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1872,10 +1824,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K26" t="b">
+        <v>0</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1929,10 +1879,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1981,10 +1929,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K28" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -2033,10 +1979,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K29" t="b">
+        <v>0</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2090,10 +2034,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K30" t="b">
+        <v>0</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -2147,10 +2089,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K31" t="b">
+        <v>0</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2204,10 +2144,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K32" t="b">
+        <v>0</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2261,10 +2199,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K33" t="b">
+        <v>0</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2318,10 +2254,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K34" t="b">
+        <v>0</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2375,10 +2309,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K35" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2427,10 +2359,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K36" t="b">
+        <v>0</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2484,10 +2414,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -2536,10 +2464,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K38" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2588,10 +2514,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K39" t="b">
+        <v>0</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2645,10 +2569,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K40" t="b">
+        <v>0</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2702,10 +2624,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K41" t="b">
+        <v>0</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2759,10 +2679,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K42" t="b">
+        <v>0</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2816,10 +2734,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K43" t="b">
+        <v>0</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2873,10 +2789,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K44" t="b">
+        <v>0</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2930,10 +2844,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K45" t="b">
+        <v>0</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2987,10 +2899,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K46" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3039,10 +2949,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K47" t="b">
+        <v>0</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -3096,10 +3004,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K48" t="b">
+        <v>0</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -3153,10 +3059,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K49" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3205,10 +3109,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K50" t="b">
+        <v>0</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -3262,10 +3164,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K51" t="b">
+        <v>0</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -3319,10 +3219,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K52" t="b">
+        <v>0</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -3376,10 +3274,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K53" t="b">
+        <v>0</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -3433,10 +3329,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K54" t="b">
+        <v>0</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3490,10 +3384,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K55" t="b">
+        <v>0</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -3547,10 +3439,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K56" t="b">
+        <v>0</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -3604,10 +3494,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K57" t="b">
+        <v>0</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -3661,10 +3549,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K58" t="b">
+        <v>0</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -3718,10 +3604,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K59" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -3770,10 +3654,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K60" t="b">
+        <v>0</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -3827,10 +3709,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K61" t="b">
+        <v>0</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -3884,10 +3764,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K62" t="b">
+        <v>0</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -3946,10 +3824,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K63" t="b">
+        <v>0</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -4003,10 +3879,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K64" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -4060,10 +3934,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K65" t="b">
+        <v>0</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -4117,10 +3989,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K66" t="b">
+        <v>0</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -4174,10 +4044,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K67" t="b">
+        <v>0</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -4231,10 +4099,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K68" t="b">
+        <v>0</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -4288,10 +4154,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K69" t="b">
+        <v>0</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -4345,10 +4209,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K70" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -4397,10 +4259,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K71" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -4449,10 +4309,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -4501,10 +4359,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K73" t="b">
+        <v>0</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -4558,10 +4414,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K74" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -4610,10 +4464,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K75" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -4662,10 +4514,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K76" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -4714,10 +4564,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K77" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -4766,10 +4614,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K78" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -4818,10 +4664,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K79" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -4870,10 +4714,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K80" t="b">
+        <v>0</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -4927,10 +4769,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K81" t="b">
+        <v>0</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -4984,10 +4824,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K82" t="b">
+        <v>0</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -5041,10 +4879,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K83" t="b">
+        <v>0</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -5098,10 +4934,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K84" t="b">
+        <v>0</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -5155,10 +4989,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K85" t="b">
+        <v>0</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -5212,10 +5044,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K86" t="b">
+        <v>0</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -5269,10 +5099,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K87" t="b">
+        <v>0</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -5326,10 +5154,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K88" t="b">
+        <v>0</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -5383,10 +5209,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K89" t="b">
+        <v>0</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -5440,10 +5264,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K90" t="b">
+        <v>0</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -5497,10 +5319,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K91" t="b">
+        <v>0</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -5554,10 +5374,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K92" t="b">
+        <v>0</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -5611,10 +5429,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K93" t="b">
+        <v>0</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -5668,10 +5484,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K94" t="b">
+        <v>0</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -5730,10 +5544,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K95" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -5787,10 +5599,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K96" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -5834,10 +5644,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K97" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -5891,10 +5699,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K98" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -5943,10 +5749,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K99" t="b">
+        <v>0</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -6000,10 +5804,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K100" t="b">
+        <v>0</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
@@ -6057,10 +5859,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K101" t="b">
+        <v>0</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -6114,10 +5914,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K102" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -6166,10 +5964,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K103" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -6218,10 +6014,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K104" t="b">
+        <v>0</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
@@ -6275,10 +6069,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K105" t="b">
+        <v>0</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -6332,10 +6124,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K106" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -6384,10 +6174,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K107" t="b">
+        <v>0</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -6441,10 +6229,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K108" t="b">
+        <v>0</v>
       </c>
       <c r="L108" t="inlineStr">
         <is>
@@ -6498,10 +6284,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K109" t="b">
+        <v>0</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -6555,10 +6339,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K110" t="b">
+        <v>0</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -6612,10 +6394,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K111" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -6664,10 +6444,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K112" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -6716,10 +6494,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K113" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -6768,10 +6544,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K114" t="b">
+        <v>0</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -6825,10 +6599,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K115" t="b">
+        <v>0</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -6882,10 +6654,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K116" t="b">
+        <v>0</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -6939,10 +6709,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K117" t="b">
+        <v>0</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -6996,10 +6764,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K118" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -7048,10 +6814,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K119" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -7100,10 +6864,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K120" t="b">
+        <v>0</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -7157,10 +6919,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K121" t="b">
+        <v>0</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -7214,10 +6974,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K122" t="b">
+        <v>0</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -7271,10 +7029,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K123" t="b">
+        <v>0</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -7328,10 +7084,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K124" t="b">
+        <v>0</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -7385,10 +7139,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K125" t="b">
+        <v>0</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -7442,10 +7194,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K126" t="b">
+        <v>0</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -7499,10 +7249,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K127" t="b">
+        <v>0</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -7561,10 +7309,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K128" t="b">
+        <v>0</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -7623,10 +7369,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K129" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -7680,10 +7424,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K130" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -7737,10 +7479,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K131" t="b">
+        <v>0</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -7799,10 +7539,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K132" t="b">
+        <v>0</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -7856,10 +7594,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K133" t="b">
+        <v>0</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -7913,10 +7649,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K134" t="b">
+        <v>0</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
@@ -7970,10 +7704,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K135" t="b">
+        <v>0</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -8027,10 +7759,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K136" t="b">
+        <v>0</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -8084,10 +7814,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K137" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -8136,10 +7864,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K138" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -8188,10 +7914,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K139" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -8240,10 +7964,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K140" t="b">
+        <v>0</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -8297,10 +8019,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K141" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -8349,10 +8069,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K142" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -8401,10 +8119,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K143" t="b">
+        <v>0</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -8458,10 +8174,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K144" t="b">
+        <v>0</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
@@ -8515,10 +8229,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K145" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -8567,10 +8279,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K146" t="b">
+        <v>0</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -8624,10 +8334,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K147" t="b">
+        <v>0</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -8681,10 +8389,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K148" t="b">
+        <v>0</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
@@ -8738,10 +8444,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K149" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -8795,10 +8499,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K150" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -8852,10 +8554,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K151" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -8899,10 +8599,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K152" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -8951,10 +8649,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K153" t="b">
+        <v>0</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
@@ -9008,10 +8704,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K154" t="b">
+        <v>0</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -9065,10 +8759,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K155" t="b">
+        <v>0</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -9122,10 +8814,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K156" t="b">
+        <v>0</v>
       </c>
       <c r="L156" t="inlineStr">
         <is>
@@ -9179,10 +8869,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K157" t="b">
+        <v>0</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -9236,10 +8924,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K158" t="b">
+        <v>0</v>
       </c>
       <c r="L158" t="inlineStr">
         <is>
@@ -9293,10 +8979,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K159" t="b">
+        <v>0</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -9350,10 +9034,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K160" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -9402,10 +9084,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K161" t="b">
+        <v>0</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -9459,10 +9139,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K162" t="b">
+        <v>0</v>
       </c>
       <c r="L162" t="inlineStr">
         <is>
@@ -9516,10 +9194,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K163" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -9568,10 +9244,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K164" t="b">
+        <v>0</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -9625,10 +9299,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K165" t="b">
+        <v>0</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -9682,10 +9354,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K166" t="b">
+        <v>0</v>
       </c>
       <c r="L166" t="inlineStr">
         <is>
@@ -9739,10 +9409,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K167" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -9791,10 +9459,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K168" t="b">
+        <v>0</v>
       </c>
       <c r="L168" t="inlineStr">
         <is>
@@ -9848,10 +9514,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K169" t="b">
+        <v>0</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -9905,10 +9569,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K170" t="b">
+        <v>0</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -9962,10 +9624,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K171" t="b">
+        <v>0</v>
       </c>
       <c r="L171" t="inlineStr">
         <is>
@@ -10019,10 +9679,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K172" t="b">
+        <v>0</v>
       </c>
       <c r="L172" t="inlineStr">
         <is>
@@ -10076,10 +9734,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K173" t="b">
+        <v>0</v>
       </c>
       <c r="L173" t="inlineStr">
         <is>
@@ -10133,10 +9789,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K174" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -10185,10 +9839,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K175" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="176">
@@ -10237,10 +9889,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K176" t="b">
+        <v>0</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -10294,10 +9944,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K177" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -10346,10 +9994,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K178" t="b">
+        <v>0</v>
       </c>
       <c r="L178" t="inlineStr">
         <is>
@@ -10403,10 +10049,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K179" t="b">
+        <v>0</v>
       </c>
       <c r="L179" t="inlineStr">
         <is>
@@ -10460,10 +10104,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K180" t="b">
+        <v>0</v>
       </c>
       <c r="L180" t="inlineStr">
         <is>
@@ -10517,10 +10159,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K181" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K181" t="b">
+        <v>0</v>
       </c>
       <c r="L181" t="inlineStr">
         <is>
@@ -10574,10 +10214,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K182" t="b">
+        <v>0</v>
       </c>
       <c r="L182" t="inlineStr">
         <is>
@@ -10631,10 +10269,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K183" t="b">
+        <v>0</v>
       </c>
       <c r="L183" t="inlineStr">
         <is>
@@ -10688,10 +10324,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K184" t="b">
+        <v>0</v>
       </c>
       <c r="L184" t="inlineStr">
         <is>
@@ -10745,10 +10379,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K185" t="b">
+        <v>0</v>
       </c>
       <c r="L185" t="inlineStr">
         <is>
@@ -10802,10 +10434,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K186" t="b">
+        <v>0</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -10859,10 +10489,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K187" t="b">
+        <v>0</v>
       </c>
       <c r="L187" t="inlineStr">
         <is>
@@ -10916,10 +10544,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K188" t="b">
+        <v>0</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -10973,10 +10599,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K189" t="b">
+        <v>0</v>
       </c>
       <c r="L189" t="inlineStr">
         <is>
@@ -11030,10 +10654,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K190" t="b">
+        <v>0</v>
       </c>
       <c r="L190" t="inlineStr">
         <is>
@@ -11087,10 +10709,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K191" t="b">
+        <v>0</v>
       </c>
       <c r="L191" t="inlineStr">
         <is>
@@ -11144,10 +10764,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K192" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -11196,10 +10814,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K193" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K193" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="194">
@@ -11248,10 +10864,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K194" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K194" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="195">
@@ -11300,10 +10914,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K195" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K195" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="196">
@@ -11352,10 +10964,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K196" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K196" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="197">
@@ -11404,10 +11014,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K197" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K197" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -11456,10 +11064,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K198" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K198" t="b">
+        <v>0</v>
       </c>
       <c r="L198" t="inlineStr">
         <is>
@@ -11513,10 +11119,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K199" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K199" t="b">
+        <v>0</v>
       </c>
       <c r="L199" t="inlineStr">
         <is>
@@ -11570,10 +11174,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K200" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K200" t="b">
+        <v>0</v>
       </c>
       <c r="L200" t="inlineStr">
         <is>
@@ -11627,10 +11229,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K201" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K201" t="b">
+        <v>0</v>
       </c>
       <c r="L201" t="inlineStr">
         <is>
@@ -11684,10 +11284,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K202" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K202" t="b">
+        <v>0</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -11741,10 +11339,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K203" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K203" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="204">
@@ -11793,10 +11389,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K204" t="b">
+        <v>0</v>
       </c>
       <c r="L204" t="inlineStr">
         <is>
@@ -11850,10 +11444,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K205" t="b">
+        <v>0</v>
       </c>
       <c r="L205" t="inlineStr">
         <is>
@@ -11907,10 +11499,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K206" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K206" t="b">
+        <v>0</v>
       </c>
       <c r="L206" t="inlineStr">
         <is>
@@ -11964,10 +11554,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K207" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K207" t="b">
+        <v>0</v>
       </c>
       <c r="L207" t="inlineStr">
         <is>
@@ -12021,10 +11609,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K208" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="209">
@@ -12073,10 +11659,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K209" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="210">
@@ -12125,10 +11709,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K210" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K210" t="b">
+        <v>0</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
@@ -12182,10 +11764,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K211" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K211" t="b">
+        <v>0</v>
       </c>
       <c r="L211" t="inlineStr">
         <is>
@@ -12239,10 +11819,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K212" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K212" t="b">
+        <v>0</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -12296,10 +11874,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K213" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K213" t="b">
+        <v>0</v>
       </c>
       <c r="L213" t="inlineStr">
         <is>
@@ -12353,10 +11929,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K214" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K214" t="b">
+        <v>0</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -12410,10 +11984,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K215" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K215" t="b">
+        <v>0</v>
       </c>
       <c r="L215" t="inlineStr">
         <is>
@@ -12467,10 +12039,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K216" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K216" t="b">
+        <v>0</v>
       </c>
       <c r="L216" t="inlineStr">
         <is>
@@ -12524,10 +12094,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K217" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K217" t="b">
+        <v>0</v>
       </c>
       <c r="L217" t="inlineStr">
         <is>
@@ -12581,10 +12149,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K218" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K218" t="b">
+        <v>0</v>
       </c>
       <c r="L218" t="inlineStr">
         <is>
@@ -12638,10 +12204,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K219" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K219" t="b">
+        <v>0</v>
       </c>
       <c r="L219" t="inlineStr">
         <is>
@@ -12695,10 +12259,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K220" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K220" t="b">
+        <v>0</v>
       </c>
       <c r="L220" t="inlineStr">
         <is>
@@ -12752,10 +12314,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K221" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K221" t="b">
+        <v>0</v>
       </c>
       <c r="L221" t="inlineStr">
         <is>
@@ -12809,10 +12369,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K222" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K222" t="b">
+        <v>0</v>
       </c>
       <c r="L222" t="inlineStr">
         <is>
@@ -12866,10 +12424,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K223" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K223" t="b">
+        <v>0</v>
       </c>
       <c r="L223" t="inlineStr">
         <is>
@@ -12923,10 +12479,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K224" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K224" t="b">
+        <v>0</v>
       </c>
       <c r="L224" t="inlineStr">
         <is>
@@ -12980,10 +12534,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K225" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K225" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="226">
@@ -13032,10 +12584,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K226" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K226" t="b">
+        <v>0</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -13089,10 +12639,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K227" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K227" t="b">
+        <v>0</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -13146,10 +12694,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K228" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K228" t="b">
+        <v>0</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -13203,10 +12749,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K229" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K229" t="b">
+        <v>0</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -13265,10 +12809,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K230" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K230" t="b">
+        <v>0</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -13327,10 +12869,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K231" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K231" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="232">
@@ -13384,10 +12924,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K232" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K232" t="b">
+        <v>0</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -13446,10 +12984,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K233" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K233" t="b">
+        <v>0</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -13508,10 +13044,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K234" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K234" t="b">
+        <v>0</v>
       </c>
       <c r="L234" t="inlineStr">
         <is>
@@ -13570,10 +13104,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K235" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K235" t="b">
+        <v>0</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -13632,10 +13164,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K236" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K236" t="b">
+        <v>0</v>
       </c>
       <c r="L236" t="inlineStr">
         <is>
@@ -13694,10 +13224,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K237" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K237" t="b">
+        <v>0</v>
       </c>
       <c r="L237" t="inlineStr">
         <is>
@@ -13746,10 +13274,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K238" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K238" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="239">
@@ -13798,10 +13324,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K239" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K239" t="b">
+        <v>0</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -13855,10 +13379,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K240" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K240" t="b">
+        <v>0</v>
       </c>
       <c r="L240" t="inlineStr">
         <is>
@@ -13912,10 +13434,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K241" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K241" t="b">
+        <v>0</v>
       </c>
       <c r="L241" t="inlineStr">
         <is>
@@ -13969,10 +13489,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K242" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K242" t="b">
+        <v>0</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -14026,10 +13544,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K243" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K243" t="b">
+        <v>0</v>
       </c>
       <c r="L243" t="inlineStr">
         <is>
@@ -14083,10 +13599,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K244" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K244" t="b">
+        <v>0</v>
       </c>
       <c r="L244" t="inlineStr">
         <is>
@@ -14140,10 +13654,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K245" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K245" t="b">
+        <v>0</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -14197,10 +13709,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K246" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K246" t="b">
+        <v>0</v>
       </c>
       <c r="L246" t="inlineStr">
         <is>
@@ -14254,10 +13764,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K247" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K247" t="b">
+        <v>0</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -14311,10 +13819,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K248" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K248" t="b">
+        <v>0</v>
       </c>
       <c r="L248" t="inlineStr">
         <is>
@@ -14368,10 +13874,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K249" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K249" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="250">
@@ -14420,10 +13924,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K250" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K250" t="b">
+        <v>0</v>
       </c>
       <c r="L250" t="inlineStr">
         <is>
@@ -14477,10 +13979,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K251" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K251" t="b">
+        <v>0</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -14534,10 +14034,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K252" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K252" t="b">
+        <v>0</v>
       </c>
       <c r="L252" t="inlineStr">
         <is>
@@ -14591,10 +14089,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K253" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K253" t="b">
+        <v>0</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -14648,10 +14144,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K254" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K254" t="b">
+        <v>0</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -14710,10 +14204,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K255" t="b">
+        <v>0</v>
       </c>
       <c r="L255" t="inlineStr">
         <is>
@@ -14767,10 +14259,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K256" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K256" t="b">
+        <v>0</v>
       </c>
       <c r="L256" t="inlineStr">
         <is>
@@ -14824,10 +14314,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K257" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K257" t="b">
+        <v>0</v>
       </c>
       <c r="L257" t="inlineStr">
         <is>
@@ -14881,10 +14369,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K258" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K258" t="b">
+        <v>0</v>
       </c>
       <c r="L258" t="inlineStr">
         <is>
@@ -14938,10 +14424,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K259" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K259" t="b">
+        <v>0</v>
       </c>
       <c r="L259" t="inlineStr">
         <is>
@@ -14995,10 +14479,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K260" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K260" t="b">
+        <v>0</v>
       </c>
       <c r="L260" t="inlineStr">
         <is>
@@ -15052,10 +14534,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K261" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K261" t="b">
+        <v>0</v>
       </c>
       <c r="L261" t="inlineStr">
         <is>
@@ -15109,10 +14589,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K262" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K262" t="b">
+        <v>0</v>
       </c>
       <c r="L262" t="inlineStr">
         <is>
@@ -15166,10 +14644,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K263" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K263" t="b">
+        <v>0</v>
       </c>
       <c r="L263" t="inlineStr">
         <is>
@@ -15223,10 +14699,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K264" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K264" t="b">
+        <v>0</v>
       </c>
       <c r="L264" t="inlineStr">
         <is>
@@ -15280,10 +14754,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K265" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K265" t="b">
+        <v>0</v>
       </c>
       <c r="L265" t="inlineStr">
         <is>
@@ -15337,10 +14809,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K266" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K266" t="b">
+        <v>0</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -15394,10 +14864,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K267" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K267" t="b">
+        <v>0</v>
       </c>
       <c r="L267" t="inlineStr">
         <is>
@@ -15451,10 +14919,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K268" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K268" t="b">
+        <v>0</v>
       </c>
       <c r="L268" t="inlineStr">
         <is>
@@ -15508,10 +14974,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K269" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K269" t="b">
+        <v>0</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -15565,10 +15029,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K270" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K270" t="b">
+        <v>0</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -15622,10 +15084,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K271" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K271" t="b">
+        <v>0</v>
       </c>
       <c r="L271" t="inlineStr">
         <is>
@@ -15679,10 +15139,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K272" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K272" t="b">
+        <v>0</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -15736,10 +15194,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K273" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K273" t="b">
+        <v>0</v>
       </c>
       <c r="L273" t="inlineStr">
         <is>
@@ -15793,10 +15249,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K274" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K274" t="b">
+        <v>0</v>
       </c>
       <c r="L274" t="inlineStr">
         <is>
@@ -15850,10 +15304,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K275" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K275" t="b">
+        <v>0</v>
       </c>
       <c r="L275" t="inlineStr">
         <is>
@@ -15907,10 +15359,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K276" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K276" t="b">
+        <v>0</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -15964,10 +15414,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K277" t="b">
+        <v>0</v>
       </c>
       <c r="L277" t="inlineStr">
         <is>
@@ -16021,10 +15469,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K278" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K278" t="b">
+        <v>0</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -16078,10 +15524,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K279" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K279" t="b">
+        <v>0</v>
       </c>
       <c r="L279" t="inlineStr">
         <is>
@@ -16135,10 +15579,8 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K280" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K280" t="b">
+        <v>0</v>
       </c>
       <c r="L280" t="inlineStr">
         <is>
@@ -16187,10 +15629,8 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K281" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K281" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="282">
@@ -16234,16 +15674,14 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K282" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K282" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -16288,7 +15726,7 @@
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE (2026-08-04 00:45)</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
@@ -16300,7 +15738,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -16345,7 +15783,7 @@
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE (2026-08-04 00:45)</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
@@ -16357,7 +15795,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -16402,7 +15840,7 @@
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE (2026-08-04 00:45)</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
@@ -16457,10 +15895,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K286" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K286" t="b">
+        <v>0</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -16514,10 +15950,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K287" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K287" t="b">
+        <v>0</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -16571,10 +16005,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K288" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K288" t="b">
+        <v>0</v>
       </c>
       <c r="L288" t="inlineStr">
         <is>
@@ -16628,10 +16060,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K289" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K289" t="b">
+        <v>0</v>
       </c>
       <c r="L289" t="inlineStr">
         <is>
@@ -16685,10 +16115,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K290" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K290" t="b">
+        <v>0</v>
       </c>
       <c r="L290" t="inlineStr">
         <is>
@@ -16742,10 +16170,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K291" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K291" t="b">
+        <v>0</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -16799,10 +16225,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K292" t="b">
+        <v>0</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -16856,10 +16280,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K293" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K293" t="b">
+        <v>0</v>
       </c>
       <c r="L293" t="inlineStr">
         <is>
@@ -16913,10 +16335,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K294" t="b">
+        <v>0</v>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -16970,10 +16390,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K295" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K295" t="b">
+        <v>0</v>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -17027,10 +16445,8 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K296" t="b">
+        <v>0</v>
       </c>
       <c r="L296" t="inlineStr">
         <is>
@@ -17084,10 +16500,8 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K297" t="b">
+        <v>0</v>
       </c>
       <c r="L297" t="inlineStr">
         <is>
@@ -17141,10 +16555,8 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K298" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K298" t="b">
+        <v>0</v>
       </c>
       <c r="L298" t="inlineStr">
         <is>
@@ -17198,10 +16610,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K299" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K299" t="b">
+        <v>0</v>
       </c>
       <c r="L299" t="inlineStr">
         <is>
@@ -17255,10 +16665,8 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K300" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K300" t="b">
+        <v>0</v>
       </c>
       <c r="L300" t="inlineStr">
         <is>
@@ -17312,10 +16720,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K301" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K301" t="b">
+        <v>0</v>
       </c>
       <c r="L301" t="inlineStr">
         <is>
@@ -17369,10 +16775,8 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K302" t="b">
+        <v>0</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -17426,10 +16830,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K303" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K303" t="b">
+        <v>0</v>
       </c>
       <c r="L303" t="inlineStr">
         <is>
@@ -17483,10 +16885,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K304" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K304" t="b">
+        <v>0</v>
       </c>
       <c r="L304" t="inlineStr">
         <is>
@@ -17540,10 +16940,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K305" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K305" t="b">
+        <v>0</v>
       </c>
       <c r="L305" t="inlineStr">
         <is>
@@ -17597,10 +16995,8 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K306" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K306" t="b">
+        <v>0</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -17654,10 +17050,8 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K307" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K307" t="b">
+        <v>0</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -17711,10 +17105,8 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K308" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K308" t="b">
+        <v>0</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -17768,10 +17160,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K309" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K309" t="b">
+        <v>0</v>
       </c>
       <c r="L309" t="inlineStr">
         <is>
@@ -17825,10 +17215,8 @@
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="K310" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K310" t="b">
+        <v>0</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -17882,10 +17270,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K311" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K311" t="b">
+        <v>0</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -17939,10 +17325,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K312" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K312" t="b">
+        <v>0</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -17996,10 +17380,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K313" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K313" t="b">
+        <v>0</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -18053,10 +17435,8 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K314" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K314" t="b">
+        <v>0</v>
       </c>
       <c r="L314" t="inlineStr">
         <is>
@@ -18110,10 +17490,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K315" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K315" t="b">
+        <v>0</v>
       </c>
       <c r="L315" t="inlineStr">
         <is>
@@ -18167,10 +17545,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K316" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K316" t="b">
+        <v>0</v>
       </c>
       <c r="L316" t="inlineStr">
         <is>
@@ -18224,10 +17600,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K317" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K317" t="b">
+        <v>0</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -18281,10 +17655,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K318" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K318" t="b">
+        <v>0</v>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -18338,10 +17710,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K319" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K319" t="b">
+        <v>0</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -18395,10 +17765,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K320" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K320" t="b">
+        <v>0</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -18452,10 +17820,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K321" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K321" t="b">
+        <v>0</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -18509,10 +17875,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K322" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K322" t="b">
+        <v>0</v>
       </c>
       <c r="L322" t="inlineStr">
         <is>
@@ -18566,10 +17930,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K323" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K323" t="b">
+        <v>0</v>
       </c>
       <c r="L323" t="inlineStr">
         <is>
@@ -18623,10 +17985,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K324" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K324" t="b">
+        <v>0</v>
       </c>
       <c r="L324" t="inlineStr">
         <is>
@@ -18680,10 +18040,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K325" t="b">
+        <v>0</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -18737,10 +18095,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K326" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K326" t="b">
+        <v>0</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -18794,10 +18150,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K327" t="b">
+        <v>0</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -18851,10 +18205,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K328" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K328" t="b">
+        <v>0</v>
       </c>
       <c r="L328" t="inlineStr">
         <is>
@@ -18908,10 +18260,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K329" t="b">
+        <v>0</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -18965,10 +18315,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K330" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K330" t="b">
+        <v>0</v>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -19022,10 +18370,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K331" t="b">
+        <v>0</v>
       </c>
       <c r="L331" t="inlineStr">
         <is>
@@ -19079,10 +18425,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K332" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K332" t="b">
+        <v>0</v>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -19136,10 +18480,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K333" t="b">
+        <v>0</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -19193,10 +18535,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K334" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K334" t="b">
+        <v>0</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -19250,10 +18590,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K335" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K335" t="b">
+        <v>0</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -19307,10 +18645,8 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K336" t="b">
+        <v>0</v>
       </c>
       <c r="L336" t="inlineStr">
         <is>
@@ -19364,10 +18700,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K337" t="b">
+        <v>0</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -19421,10 +18755,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K338" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K338" t="b">
+        <v>0</v>
       </c>
       <c r="L338" t="inlineStr">
         <is>
@@ -19478,10 +18810,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K339" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K339" t="b">
+        <v>0</v>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -19535,10 +18865,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K340" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K340" t="b">
+        <v>0</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -19592,10 +18920,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K341" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K341" t="b">
+        <v>0</v>
       </c>
       <c r="L341" t="inlineStr">
         <is>
@@ -19649,10 +18975,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K342" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K342" t="b">
+        <v>0</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -19706,10 +19030,8 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K343" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="K343" t="b">
+        <v>0</v>
       </c>
       <c r="L343" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update HPR UK Turkey application status
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -7771,7 +7771,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>🔥 HOT LEAD (APPLIED)</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7814,8 +7814,10 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K137" t="b">
-        <v>0</v>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 08:54)</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -15852,7 +15854,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -15895,8 +15897,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K286" t="b">
-        <v>0</v>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 00:54)</t>
+        </is>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -15907,7 +15911,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -15950,8 +15954,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K287" t="b">
-        <v>0</v>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 00:58)</t>
+        </is>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -15962,7 +15968,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -16005,8 +16011,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K288" t="b">
-        <v>0</v>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:05)</t>
+        </is>
       </c>
       <c r="L288" t="inlineStr">
         <is>
@@ -16017,7 +16025,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -16060,8 +16068,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K289" t="b">
-        <v>0</v>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:11)</t>
+        </is>
       </c>
       <c r="L289" t="inlineStr">
         <is>
@@ -16072,7 +16082,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -16115,8 +16125,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K290" t="b">
-        <v>0</v>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:16)</t>
+        </is>
       </c>
       <c r="L290" t="inlineStr">
         <is>
@@ -16127,7 +16139,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -16170,8 +16182,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K291" t="b">
-        <v>0</v>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:20)</t>
+        </is>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -16182,7 +16196,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -16225,8 +16239,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K292" t="b">
-        <v>0</v>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:30)</t>
+        </is>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -16237,7 +16253,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -16280,8 +16296,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K293" t="b">
-        <v>0</v>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:35)</t>
+        </is>
       </c>
       <c r="L293" t="inlineStr">
         <is>
@@ -16292,7 +16310,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -16335,8 +16353,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K294" t="b">
-        <v>0</v>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:42)</t>
+        </is>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -16347,7 +16367,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -16390,8 +16410,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K295" t="b">
-        <v>0</v>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:46)</t>
+        </is>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -16457,7 +16479,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -16500,8 +16522,10 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K297" t="b">
-        <v>0</v>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:52)</t>
+        </is>
       </c>
       <c r="L297" t="inlineStr">
         <is>
@@ -16512,7 +16536,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -16555,8 +16579,10 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K298" t="b">
-        <v>0</v>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 01:59)</t>
+        </is>
       </c>
       <c r="L298" t="inlineStr">
         <is>
@@ -16567,7 +16593,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -16610,8 +16636,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K299" t="b">
-        <v>0</v>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:05)</t>
+        </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
@@ -16622,7 +16650,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -16665,8 +16693,10 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K300" t="b">
-        <v>0</v>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:10)</t>
+        </is>
       </c>
       <c r="L300" t="inlineStr">
         <is>
@@ -16677,7 +16707,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -16720,8 +16750,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K301" t="b">
-        <v>0</v>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:16)</t>
+        </is>
       </c>
       <c r="L301" t="inlineStr">
         <is>
@@ -16732,7 +16764,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -16775,8 +16807,10 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K302" t="b">
-        <v>0</v>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:22)</t>
+        </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -16787,7 +16821,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -16830,8 +16864,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K303" t="b">
-        <v>0</v>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:26)</t>
+        </is>
       </c>
       <c r="L303" t="inlineStr">
         <is>
@@ -16842,7 +16878,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -16885,8 +16921,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K304" t="b">
-        <v>0</v>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:31)</t>
+        </is>
       </c>
       <c r="L304" t="inlineStr">
         <is>
@@ -16897,7 +16935,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -16940,8 +16978,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K305" t="b">
-        <v>0</v>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:37)</t>
+        </is>
       </c>
       <c r="L305" t="inlineStr">
         <is>
@@ -16952,7 +16992,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -16995,8 +17035,10 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K306" t="b">
-        <v>0</v>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:41)</t>
+        </is>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -17007,7 +17049,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -17050,8 +17092,10 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K307" t="b">
-        <v>0</v>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:46)</t>
+        </is>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -17062,7 +17106,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -17105,8 +17149,10 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K308" t="b">
-        <v>0</v>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:50)</t>
+        </is>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -17117,7 +17163,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -17160,8 +17206,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K309" t="b">
-        <v>0</v>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 02:55)</t>
+        </is>
       </c>
       <c r="L309" t="inlineStr">
         <is>
@@ -17172,7 +17220,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -17215,8 +17263,10 @@
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="K310" t="b">
-        <v>0</v>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:01)</t>
+        </is>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -17227,7 +17277,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -17270,8 +17320,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K311" t="b">
-        <v>0</v>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:06)</t>
+        </is>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -17282,7 +17334,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -17325,8 +17377,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K312" t="b">
-        <v>0</v>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:12)</t>
+        </is>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -17337,7 +17391,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -17380,8 +17434,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K313" t="b">
-        <v>0</v>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:18)</t>
+        </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -17392,7 +17448,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -17435,8 +17491,10 @@
           <t>Facebook Group</t>
         </is>
       </c>
-      <c r="K314" t="b">
-        <v>0</v>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:22)</t>
+        </is>
       </c>
       <c r="L314" t="inlineStr">
         <is>
@@ -17447,7 +17505,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -17490,8 +17548,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K315" t="b">
-        <v>0</v>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:28)</t>
+        </is>
       </c>
       <c r="L315" t="inlineStr">
         <is>
@@ -17502,7 +17562,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -17545,8 +17605,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K316" t="b">
-        <v>0</v>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:34)</t>
+        </is>
       </c>
       <c r="L316" t="inlineStr">
         <is>
@@ -17557,7 +17619,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -17600,8 +17662,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K317" t="b">
-        <v>0</v>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:39)</t>
+        </is>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -17612,7 +17676,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -17655,8 +17719,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K318" t="b">
-        <v>0</v>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:45)</t>
+        </is>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -17667,7 +17733,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -17710,8 +17776,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K319" t="b">
-        <v>0</v>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:51)</t>
+        </is>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -17722,7 +17790,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -17765,8 +17833,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K320" t="b">
-        <v>0</v>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 03:58)</t>
+        </is>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -17777,7 +17847,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -17820,8 +17890,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K321" t="b">
-        <v>0</v>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:04)</t>
+        </is>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -17832,7 +17904,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -17875,8 +17947,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K322" t="b">
-        <v>0</v>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:09)</t>
+        </is>
       </c>
       <c r="L322" t="inlineStr">
         <is>
@@ -17887,7 +17961,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -17930,8 +18004,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K323" t="b">
-        <v>0</v>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:14)</t>
+        </is>
       </c>
       <c r="L323" t="inlineStr">
         <is>
@@ -17942,7 +18018,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -17985,8 +18061,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K324" t="b">
-        <v>0</v>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:18)</t>
+        </is>
       </c>
       <c r="L324" t="inlineStr">
         <is>
@@ -17997,7 +18075,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -18040,8 +18118,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K325" t="b">
-        <v>0</v>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:23)</t>
+        </is>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -18052,7 +18132,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -18095,8 +18175,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K326" t="b">
-        <v>0</v>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:29)</t>
+        </is>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -18107,7 +18189,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -18150,8 +18232,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K327" t="b">
-        <v>0</v>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:34)</t>
+        </is>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -18162,7 +18246,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -18205,8 +18289,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K328" t="b">
-        <v>0</v>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:40)</t>
+        </is>
       </c>
       <c r="L328" t="inlineStr">
         <is>
@@ -18217,7 +18303,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -18260,8 +18346,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K329" t="b">
-        <v>0</v>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:44)</t>
+        </is>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -18272,7 +18360,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -18315,8 +18403,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K330" t="b">
-        <v>0</v>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:50)</t>
+        </is>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -18327,7 +18417,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -18370,8 +18460,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K331" t="b">
-        <v>0</v>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 04:56)</t>
+        </is>
       </c>
       <c r="L331" t="inlineStr">
         <is>
@@ -18382,7 +18474,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -18425,8 +18517,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K332" t="b">
-        <v>0</v>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:00)</t>
+        </is>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -18437,7 +18531,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -18480,8 +18574,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K333" t="b">
-        <v>0</v>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:04)</t>
+        </is>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -18492,7 +18588,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -18535,8 +18631,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K334" t="b">
-        <v>0</v>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:11)</t>
+        </is>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -18547,7 +18645,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -18590,8 +18688,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K335" t="b">
-        <v>0</v>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:17)</t>
+        </is>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -18602,7 +18702,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -18645,8 +18745,10 @@
           <t>Facebook Group + Enriched</t>
         </is>
       </c>
-      <c r="K336" t="b">
-        <v>0</v>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:22)</t>
+        </is>
       </c>
       <c r="L336" t="inlineStr">
         <is>
@@ -18657,7 +18759,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -18700,8 +18802,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K337" t="b">
-        <v>0</v>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:28)</t>
+        </is>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -18712,7 +18816,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -18755,8 +18859,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K338" t="b">
-        <v>0</v>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:32)</t>
+        </is>
       </c>
       <c r="L338" t="inlineStr">
         <is>
@@ -18767,7 +18873,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -18810,8 +18916,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K339" t="b">
-        <v>0</v>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:39)</t>
+        </is>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -18822,7 +18930,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -18865,8 +18973,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K340" t="b">
-        <v>0</v>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:43)</t>
+        </is>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -18877,7 +18987,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -18920,8 +19030,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K341" t="b">
-        <v>0</v>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 05:49)</t>
+        </is>
       </c>
       <c r="L341" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Diane HPR UK reply status in CRM
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -636,7 +636,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -679,8 +679,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K5" t="b">
-        <v>0</v>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 09:51)</t>
+        </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -691,7 +693,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -734,8 +736,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K6" t="b">
-        <v>0</v>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 10:05)</t>
+        </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -746,7 +750,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -789,8 +793,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K7" t="b">
-        <v>0</v>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 10:15)</t>
+        </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -801,7 +807,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -844,8 +850,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K8" t="b">
-        <v>0</v>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 10:27)</t>
+        </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -856,7 +864,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -899,8 +907,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K9" t="b">
-        <v>0</v>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 10:39)</t>
+        </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -911,7 +921,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -954,14 +964,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K10" t="b">
-        <v>0</v>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 10:53)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1004,8 +1016,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K11" t="b">
-        <v>0</v>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 11:07)</t>
+        </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1016,7 +1030,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1059,8 +1073,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K12" t="b">
-        <v>0</v>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 11:19)</t>
+        </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1071,7 +1087,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1114,8 +1130,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K13" t="b">
-        <v>0</v>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 11:34)</t>
+        </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1126,7 +1144,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1169,8 +1187,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K14" t="b">
-        <v>0</v>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 11:43)</t>
+        </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1181,7 +1201,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1224,14 +1244,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K15" t="b">
-        <v>0</v>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 11:55)</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1274,8 +1296,10 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K16" t="b">
-        <v>0</v>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 12:05)</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -7771,7 +7795,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD (APPLIED)</t>
+          <t>💬 REPLIED</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7816,7 +7840,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 08:54)</t>
+          <t>TRUE (2026-08-05 01:11)</t>
         </is>
       </c>
     </row>
@@ -16424,7 +16448,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -16467,8 +16491,10 @@
           <t>Web Search + Enriched</t>
         </is>
       </c>
-      <c r="K296" t="b">
-        <v>0</v>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 09:13)</t>
+        </is>
       </c>
       <c r="L296" t="inlineStr">
         <is>
@@ -19044,7 +19070,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -19087,8 +19113,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K342" t="b">
-        <v>0</v>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 09:25)</t>
+        </is>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -19099,7 +19127,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -19142,8 +19170,10 @@
           <t>LinkedIn Post + Enriched</t>
         </is>
       </c>
-      <c r="K343" t="b">
-        <v>0</v>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-04 09:39)</t>
+        </is>
       </c>
       <c r="L343" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update bounced emails status in CRM
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -693,7 +693,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 10:05)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -750,7 +750,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 10:15)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -15821,7 +15821,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 00:45)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
@@ -16163,7 +16163,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -16208,7 +16208,7 @@
       </c>
       <c r="K291" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 01:20)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L291" t="inlineStr">
@@ -16391,7 +16391,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="K295" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 01:46)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L295" t="inlineStr">
@@ -16562,7 +16562,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 01:59)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
@@ -16790,7 +16790,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 02:22)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
@@ -17018,7 +17018,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -17063,7 +17063,7 @@
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 02:41)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L306" t="inlineStr">
@@ -17474,7 +17474,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>❌ INVALID / BOUNCED</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -17519,7 +17519,7 @@
       </c>
       <c r="K314" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 03:22)</t>
+          <t>BOUNCED</t>
         </is>
       </c>
       <c r="L314" t="inlineStr">

</xml_diff>

<commit_message>
Update auto-reply email redirects in CRM
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -15935,7 +15935,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>🔄 AUTO-REDIRECT</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -15980,7 +15980,7 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 00:58)</t>
+          <t>REDIRECTED (sparrows.careers@altrad.com)</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -16334,7 +16334,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>🔄 AUTO-REDIRECT</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -16379,7 +16379,7 @@
       </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 01:42)</t>
+          <t>REDIRECTED (amustafa@tectonicengineering.com)</t>
         </is>
       </c>
       <c r="L294" t="inlineStr">
@@ -18899,7 +18899,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>SENT / PENDING</t>
+          <t>🔄 AUTO-REDIRECT</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -18944,7 +18944,7 @@
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-04 05:39)</t>
+          <t>REDIRECTED (ksa.recruitment@mermaid-group.com)</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">

</xml_diff>

<commit_message>
Update Proceanic Director YH Loh application status
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -1994,7 +1994,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>🔥 HOT LEAD (APPLIED)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Subsea Contractor</t>
+          <t>Mr. YH Loh (Director)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2037,8 +2037,10 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K30" t="b">
-        <v>0</v>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 12:08)</t>
+        </is>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Update Vantris Mr Tan Meng Loon acknowledgment status
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -822,7 +822,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 10:05)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 10:15)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1389,7 +1389,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1432,8 +1432,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K19" t="b">
-        <v>0</v>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-05 23:22)</t>
+        </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1444,7 +1446,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1492,8 +1494,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K20" t="b">
-        <v>0</v>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-05 23:37)</t>
+        </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1504,7 +1508,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1552,8 +1556,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K21" t="b">
-        <v>0</v>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 00:01)</t>
+        </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1564,7 +1570,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1607,8 +1613,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K22" t="b">
-        <v>0</v>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 00:18)</t>
+        </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1619,7 +1627,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1662,8 +1670,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K23" t="b">
-        <v>0</v>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 00:39)</t>
+        </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1674,7 +1684,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1717,8 +1727,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K24" t="b">
-        <v>0</v>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 01:05)</t>
+        </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1729,7 +1741,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1772,8 +1784,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K25" t="b">
-        <v>0</v>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 01:31)</t>
+        </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1784,7 +1798,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1827,14 +1841,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K26" t="b">
-        <v>0</v>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 01:44)</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1877,8 +1893,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K27" t="b">
-        <v>0</v>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 02:06)</t>
+        </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1889,7 +1907,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1932,8 +1950,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K28" t="b">
-        <v>0</v>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 02:30)</t>
+        </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1944,7 +1964,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1987,14 +2007,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K29" t="b">
-        <v>0</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 08:48)</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>🔥 HOT LEAD (APPLIED)</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2039,14 +2061,14 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-06 12:09)</t>
+          <t>TRUE (2026-08-06 09:03)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2089,8 +2111,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K31" t="b">
-        <v>0</v>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 09:24)</t>
+        </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2101,7 +2125,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2144,8 +2168,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K32" t="b">
-        <v>0</v>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 09:43)</t>
+        </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2156,7 +2182,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2199,8 +2225,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K33" t="b">
-        <v>0</v>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 10:03)</t>
+        </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2211,7 +2239,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2254,8 +2282,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K34" t="b">
-        <v>0</v>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 10:27)</t>
+        </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2266,7 +2296,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2309,8 +2339,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K35" t="b">
-        <v>0</v>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 10:42)</t>
+        </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2321,7 +2353,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2364,8 +2396,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K36" t="b">
-        <v>0</v>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 10:59)</t>
+        </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2376,7 +2410,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2419,14 +2453,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K37" t="b">
-        <v>0</v>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 11:21)</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2469,8 +2505,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K38" t="b">
-        <v>0</v>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 11:42)</t>
+        </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2481,7 +2519,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2524,14 +2562,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K39" t="b">
-        <v>0</v>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 12:05)</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>💬 REPLIED (ACKNOWLEDGED)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2574,14 +2614,16 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K40" t="b">
-        <v>0</v>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 22:26)</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2624,8 +2666,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K41" t="b">
-        <v>0</v>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 16:18)</t>
+        </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2636,7 +2680,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2679,8 +2723,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K42" t="b">
-        <v>0</v>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 16:36)</t>
+        </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -15907,7 +15953,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>❌ INVALID / BOUNCED</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -15952,7 +15998,7 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-05 02:52)</t>
         </is>
       </c>
       <c r="L287" t="inlineStr">
@@ -16021,7 +16067,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>🔄 AUTO-REDIRECT</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -16066,7 +16112,7 @@
       </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>REDIRECTED (sparrows.careers@altrad.com)</t>
+          <t>TRUE (2026-08-04 00:58)</t>
         </is>
       </c>
       <c r="L289" t="inlineStr">
@@ -16294,7 +16340,7 @@
       </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 01:20)</t>
         </is>
       </c>
       <c r="L293" t="inlineStr">
@@ -16420,7 +16466,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>🔄 AUTO-REDIRECT</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -16465,7 +16511,7 @@
       </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>REDIRECTED (amustafa@tectonicengineering.com)</t>
+          <t>TRUE (2026-08-04 01:42)</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
@@ -16522,7 +16568,7 @@
       </c>
       <c r="K297" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 01:46)</t>
         </is>
       </c>
       <c r="L297" t="inlineStr">
@@ -16693,7 +16739,7 @@
       </c>
       <c r="K300" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 01:59)</t>
         </is>
       </c>
       <c r="L300" t="inlineStr">
@@ -16921,7 +16967,7 @@
       </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 02:22)</t>
         </is>
       </c>
       <c r="L304" t="inlineStr">
@@ -17149,7 +17195,7 @@
       </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 02:41)</t>
         </is>
       </c>
       <c r="L308" t="inlineStr">
@@ -17605,7 +17651,7 @@
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t>BOUNCED</t>
+          <t>TRUE (2026-08-04 03:22)</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
@@ -19030,7 +19076,7 @@
       </c>
       <c r="K341" t="inlineStr">
         <is>
-          <t>REDIRECTED (ksa.recruitment@mermaid-group.com)</t>
+          <t>TRUE (2026-08-04 05:39)</t>
         </is>
       </c>
       <c r="L341" t="inlineStr">

</xml_diff>

<commit_message>
Real-time dual account CRM status update
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -2616,7 +2616,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>TRUE (2026-08-06 22:27)</t>
+          <t>TRUE (2026-08-06 22:26)</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2780,8 +2780,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K43" t="b">
-        <v>0</v>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 22:28)</t>
+        </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2792,7 +2794,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2835,8 +2837,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K44" t="b">
-        <v>0</v>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 22:48)</t>
+        </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2847,7 +2851,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2890,8 +2894,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K45" t="b">
-        <v>0</v>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 23:02)</t>
+        </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2902,7 +2908,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2945,8 +2951,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K46" t="b">
-        <v>0</v>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 23:26)</t>
+        </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2957,7 +2965,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3000,8 +3008,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K47" t="b">
-        <v>0</v>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-06 23:49)</t>
+        </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -3012,7 +3022,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3055,8 +3065,10 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K48" t="b">
-        <v>0</v>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-07 00:04)</t>
+        </is>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Inject 4 new targeted ASEAN agencies and reorder queue to 80% ASEAN focus
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -3074,7 +3074,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3117,8 +3117,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K49" t="b">
-        <v>0</v>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-07 03:47)</t>
+        </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -3129,7 +3131,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3172,8 +3174,10 @@
           <t>Existing Master Database + Enriched</t>
         </is>
       </c>
-      <c r="K50" t="b">
-        <v>0</v>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-07 04:02)</t>
+        </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -3184,7 +3188,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>⏳ SENT / PENDING</t>
+          <t>SENT / PENDING</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3227,8 +3231,10 @@
           <t>Existing Master Database</t>
         </is>
       </c>
-      <c r="K51" t="b">
-        <v>0</v>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>TRUE (2026-08-07 04:25)</t>
+        </is>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Prioritize all 4 MCS Subsea contacts (hr, a.sobhy, e.seoudi, mcsinfo) to TOP OF QUEUE for Monday morning
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -10457,7 +10457,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>🔥 HOT LEAD</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -10467,12 +10467,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Subsea Contractor</t>
+          <t>Ahmed Sobhy</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Amira Mahrous Sobhy</t>
+          <t>MCS Subsea Technical Manager</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -10509,7 +10509,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>🔥 HOT LEAD</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -10519,12 +10519,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Subsea Contractor</t>
+          <t>Eslam Seoudi</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Crewing Lead / Subsea Recruiter</t>
+          <t>MCS Inspection &amp; Operations Lead</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -10561,7 +10561,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>🔥 HOT LEAD</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -10571,12 +10571,12 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Subsea Contractor</t>
+          <t>MCS Operations Management</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Crewing Lead / Subsea Recruiter</t>
+          <t>Offshore Operations Desk</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">

</xml_diff>

<commit_message>
Correct MCS PIC names from inbox records: Amira Mahrous (a.sobhy) and Esraa Seoudi (e.seoudi)
</commit_message>
<xml_diff>
--- a/Master_Subsea_Contacts_v2.xlsx
+++ b/Master_Subsea_Contacts_v2.xlsx
@@ -10467,12 +10467,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Ahmed Sobhy</t>
+          <t>Amira Mahrous</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>MCS Subsea Technical Manager</t>
+          <t>Human Capital Specialist (MCS Group)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -10519,12 +10519,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Eslam Seoudi</t>
+          <t>Esraa Seoudi</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>MCS Inspection &amp; Operations Lead</t>
+          <t>Group Human Capital Head (MCS Group)</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>MCS Operations Management</t>
+          <t>MCS Subsea Operations Management</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">

</xml_diff>